<commit_message>
Update FPR/DS-020 R3 Current flows
</commit_message>
<xml_diff>
--- a/towers/FPR/DS Provide Decision Support/DS-020/input/data/R3_CurrentFlows.xlsx
+++ b/towers/FPR/DS Provide Decision Support/DS-020/input/data/R3_CurrentFlows.xlsx
@@ -3770,7 +3770,7 @@
         <v>DS-020 Process Migration</v>
       </c>
       <c r="C5" t="str">
-        <v>Migrate Perform Product Costing and Inventory Valuation business processes and 29 integrated systems from legacy to S/4 HANA target architecture</v>
+        <v>Migrate Perform Product Costing and Inventory Valuation business processes and 26 integrated systems from legacy to S/4 HANA target architecture</v>
       </c>
       <c r="D5" t="str">
         <v>IDM 2.0 Finance</v>
@@ -3873,7 +3873,7 @@
         <v>100% flow chains validated</v>
       </c>
       <c r="C5" t="str">
-        <v>All 27 flow chains verified in target state</v>
+        <v>All 24 flow chains verified in target state</v>
       </c>
       <c r="D5" t="str">
         <v>0% (pre-migration)</v>
@@ -4315,7 +4315,7 @@
         <v>Integration</v>
       </c>
       <c r="C3" t="str">
-        <v>Validate integration patterns and middleware for high-complexity flows across 29 systems (APIGEE, BOBJ, CFIN S/4 HANA, CIBR, COMPASS...)</v>
+        <v>Validate integration patterns and middleware for high-complexity flows across 26 systems (APIGEE, Azure ADF, BOBJ, CFIN S/4, CIBR...)</v>
       </c>
       <c r="D3" t="str">
         <v>High</v>
@@ -4338,7 +4338,7 @@
         <v>Data</v>
       </c>
       <c r="C4" t="str">
-        <v>Define data ownership and classification for all 27 flow chains to satisfy Data Architecture (TOGAF D) requirements</v>
+        <v>Define data ownership and classification for all 24 flow chains to satisfy Data Architecture (TOGAF D) requirements</v>
       </c>
       <c r="D4" t="str">
         <v>Medium</v>
@@ -4361,7 +4361,7 @@
         <v>Testing</v>
       </c>
       <c r="C5" t="str">
-        <v>Develop integration test scenarios covering all 27 flow chains for FUT/SIT readiness</v>
+        <v>Develop integration test scenarios covering all 24 flow chains for FUT/SIT readiness</v>
       </c>
       <c r="D5" t="str">
         <v>High</v>

</xml_diff>